<commit_message>
updated ted-2150 file to "annotated". all "raw" ted files are ready to commenting.
</commit_message>
<xml_diff>
--- a/annotators/team/tg/cost_annotation_times.xlsx
+++ b/annotators/team/tg/cost_annotation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FB280E-6427-4C46-AA11-3D2292C108EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0FCB27-EFF7-4749-AE7E-C451615A9308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>file</t>
   </si>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>ted-mdb.1978</t>
+  </si>
+  <si>
+    <t>ted-mdb.2009</t>
+  </si>
+  <si>
+    <t>ted-mdb.2150</t>
   </si>
 </sst>
 </file>
@@ -396,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -447,7 +453,7 @@
         <v>0.75</v>
       </c>
       <c r="E3" s="3">
-        <f t="shared" ref="E3:E36" si="0">D3-C3</f>
+        <f t="shared" ref="E3:E41" si="0">D3-C3</f>
         <v>4.166666666666663E-2</v>
       </c>
     </row>
@@ -708,15 +714,33 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0.6333333333333333</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0.64930555555555558</v>
+      </c>
       <c r="E29" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.5972222222222276E-2</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C30" s="3">
+        <v>0.4548611111111111</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.47222222222222221</v>
+      </c>
       <c r="E30" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.7361111111111105E-2</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -731,26 +755,82 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E33" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="F33" s="3">
+        <f>SUM(E29:E32)</f>
+        <v>3.3333333333333381E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="3">
+        <v>0.49652777777777779</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0.51736111111111116</v>
+      </c>
       <c r="E34" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="5:5" x14ac:dyDescent="0.3">
+        <v>2.083333333333337E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C35" s="3">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0.67847222222222225</v>
+      </c>
       <c r="E35" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="5:5" x14ac:dyDescent="0.3">
+        <v>1.1805555555555625E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E36" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E37" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E38" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F38" s="3">
+        <f>SUM(E34:E38)</f>
+        <v>3.2638888888888995E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E39" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E40" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E41" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
updated preanno parcor files
</commit_message>
<xml_diff>
--- a/annotators/team/tg/cost_annotation_times.xlsx
+++ b/annotators/team/tg/cost_annotation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46A4662D-3908-4CD1-9514-AD6835593372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52B45662-7573-4086-A8AB-B916965F1745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
   <si>
     <t>file</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>abcnews.199762</t>
+  </si>
+  <si>
+    <t>an-online.de.224441</t>
   </si>
 </sst>
 </file>
@@ -849,23 +852,44 @@
         <f t="shared" si="0"/>
         <v>1.7361111111111049E-2</v>
       </c>
+      <c r="F40" s="3"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E41" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="F41" s="3">
+        <f>SUM(E40:E41)</f>
+        <v>1.7361111111111049E-2</v>
+      </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>15</v>
+      </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="3">
+        <v>0.79513888888888884</v>
+      </c>
+      <c r="D42" s="3">
+        <v>0.80555555555555558</v>
+      </c>
       <c r="E42" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.0416666666666741E-2</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E43" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
+      </c>
+      <c r="F43" s="3">
+        <f>SUM(E42:E43)</f>
+        <v>1.0416666666666741E-2</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated annotated files; first IS file done
</commit_message>
<xml_diff>
--- a/annotators/team/tg/cost_annotation_times.xlsx
+++ b/annotators/team/tg/cost_annotation_times.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52B45662-7573-4086-A8AB-B916965F1745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40CB417D-D28C-4DCB-BE5C-951D39462661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -883,13 +883,19 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C43" s="3">
+        <v>0.49652777777777779</v>
+      </c>
+      <c r="D43" s="3">
+        <v>0.50694444444444442</v>
+      </c>
       <c r="E43" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.041666666666663E-2</v>
       </c>
       <c r="F43" s="3">
         <f>SUM(E42:E43)</f>
-        <v>1.0416666666666741E-2</v>
+        <v>2.083333333333337E-2</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated annotated files and annotation times
</commit_message>
<xml_diff>
--- a/annotators/team/tg/cost_annotation_times.xlsx
+++ b/annotators/team/tg/cost_annotation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1153EE-A70C-439A-9FD1-69467E4E50F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB213262-83AE-47A0-A5AE-8F1AE0A67C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="264" yWindow="1956" windowWidth="16368" windowHeight="10836" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="16368" windowHeight="10836" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1051,21 +1051,37 @@
       <c r="B56" t="s">
         <v>9</v>
       </c>
+      <c r="C56" s="3">
+        <v>0.80555555555555558</v>
+      </c>
+      <c r="D56" s="3">
+        <v>0.83333333333333337</v>
+      </c>
       <c r="E56" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.777777777777779E-2</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C57" s="3">
+        <v>0.68402777777777779</v>
+      </c>
+      <c r="D57" s="3">
+        <v>0.69791666666666663</v>
+      </c>
       <c r="E57" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.388888888888884E-2</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E58" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
+      </c>
+      <c r="F58" s="3">
+        <f>SUM(E56:E58)</f>
+        <v>4.166666666666663E-2</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>